<commit_message>
Replace account-name credit with neutral portfolio label
- Brief meta and footer now read 'Research & Data Support — Concept Portfolio'
- Workbook Read Me sheet updated to match; research_summary.xlsx regenerated
- No personal identifiers or placeholders remain in the repository
</commit_message>
<xml_diff>
--- a/data/research_summary.xlsx
+++ b/data/research_summary.xlsx
@@ -24,11 +24,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="$#,##0.00"/>
     <numFmt numFmtId="166" formatCode="YYYY-MM-DD"/>
-    <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -39,44 +38,47 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Noto Sans SC"/>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="001B2A4A"/>
       <sz val="16"/>
     </font>
     <font>
-      <name val="Noto Sans SC"/>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Noto Sans SC"/>
+      <name val="Calibri"/>
       <color rgb="0037352F"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Noto Sans SC"/>
+      <name val="Calibri"/>
       <color rgb="008C8A84"/>
       <sz val="9"/>
     </font>
     <font>
-      <name val="Noto Sans SC"/>
+      <name val="Calibri"/>
       <color rgb="001B7D46"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Noto Sans SC"/>
+      <name val="Calibri"/>
       <color rgb="00D4820A"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Noto Sans SC"/>
+      <name val="Calibri"/>
       <color rgb="00C0392B"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Noto Sans SC"/>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="001B2A4A"/>
-      <sz val="11"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="9">
@@ -157,7 +159,7 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -166,7 +168,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -187,16 +189,16 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="9" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    <xf numFmtId="9" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -566,7 +568,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="B2:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -595,7 +597,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="38" customHeight="1">
+    <row r="5" ht="22" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Project type</t>
@@ -627,11 +629,11 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>heyjdy (GitHub) — Research &amp; Data Support</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="54" customHeight="1">
+          <t>Research &amp; Data Support — Concept Portfolio</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Fictional-data disclaimer</t>
@@ -655,7 +657,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="38" customHeight="1">
+    <row r="10" ht="22" customHeight="1">
       <c r="B10" s="4" t="inlineStr">
         <is>
           <t>Raw Data sheet</t>
@@ -703,7 +705,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="54" customHeight="1">
+    <row r="14" ht="22" customHeight="1">
       <c r="B14" s="4" t="inlineStr">
         <is>
           <t>Confidence levels</t>
@@ -727,7 +729,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="38" customHeight="1">
+    <row r="16" ht="22" customHeight="1">
       <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Normalization conventions</t>
@@ -740,7 +742,7 @@
       </c>
     </row>
     <row r="17" ht="22" customHeight="1"/>
-    <row r="18" ht="70" customHeight="1">
+    <row r="18" ht="22" customHeight="1">
       <c r="B18" s="5" t="inlineStr">
         <is>
           <t>Questions about this demo workbook: see README.md in the project folder.</t>
@@ -762,16 +764,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S26"/>
+  <dimension ref="B2:S26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
@@ -781,9 +783,9 @@
     <col width="30" customWidth="1" min="14" max="14"/>
     <col width="30" customWidth="1" min="15" max="15"/>
     <col width="30" customWidth="1" min="16" max="16"/>
-    <col width="20" customWidth="1" min="17" max="17"/>
-    <col width="27" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="21" customWidth="1" min="17" max="17"/>
+    <col width="29" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -795,7 +797,7 @@
       </c>
     </row>
     <row r="3" ht="8" customHeight="1"/>
-    <row r="4" ht="70" customHeight="1">
+    <row r="4" ht="28" customHeight="1">
       <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Company / Product</t>
@@ -887,7 +889,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="54" customHeight="1">
+    <row r="5" ht="22" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
           <t>TaskPilot Pro</t>
@@ -975,7 +977,7 @@
         <v>46249</v>
       </c>
     </row>
-    <row r="6" ht="54" customHeight="1">
+    <row r="6" ht="22" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
           <t>NoteNest</t>
@@ -1063,7 +1065,7 @@
         <v>46238</v>
       </c>
     </row>
-    <row r="7" ht="38" customHeight="1">
+    <row r="7" ht="22" customHeight="1">
       <c r="B7" s="3" t="inlineStr">
         <is>
           <t>FlowDesk</t>
@@ -1151,7 +1153,7 @@
         <v>46231</v>
       </c>
     </row>
-    <row r="8" ht="38" customHeight="1">
+    <row r="8" ht="22" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
           <t>MindMesh</t>
@@ -1239,7 +1241,7 @@
         <v>46280</v>
       </c>
     </row>
-    <row r="9" ht="38" customHeight="1">
+    <row r="9" ht="22" customHeight="1">
       <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Scheduly</t>
@@ -1323,7 +1325,7 @@
         <v>46203</v>
       </c>
     </row>
-    <row r="10" ht="54" customHeight="1">
+    <row r="10" ht="22" customHeight="1">
       <c r="B10" s="4" t="inlineStr">
         <is>
           <t>DocuFlow</t>
@@ -1411,7 +1413,7 @@
         <v>46225</v>
       </c>
     </row>
-    <row r="11" ht="38" customHeight="1">
+    <row r="11" ht="22" customHeight="1">
       <c r="B11" s="3" t="inlineStr">
         <is>
           <t>TeamSync</t>
@@ -1495,7 +1497,7 @@
         <v>46161</v>
       </c>
     </row>
-    <row r="12" ht="38" customHeight="1">
+    <row r="12" ht="22" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
           <t>FocusForge</t>
@@ -1583,7 +1585,7 @@
         <v>46236</v>
       </c>
     </row>
-    <row r="13" ht="38" customHeight="1">
+    <row r="13" ht="22" customHeight="1">
       <c r="B13" s="3" t="inlineStr">
         <is>
           <t>InBoxZero</t>
@@ -1667,7 +1669,7 @@
         <v>46266</v>
       </c>
     </row>
-    <row r="14" ht="38" customHeight="1">
+    <row r="14" ht="22" customHeight="1">
       <c r="B14" s="4" t="inlineStr">
         <is>
           <t>MeetMate</t>
@@ -1751,7 +1753,7 @@
         <v>46255</v>
       </c>
     </row>
-    <row r="15" ht="38" customHeight="1">
+    <row r="15" ht="22" customHeight="1">
       <c r="B15" s="3" t="inlineStr">
         <is>
           <t>PlanCraft</t>
@@ -1835,7 +1837,7 @@
         <v>46214</v>
       </c>
     </row>
-    <row r="16" ht="38" customHeight="1">
+    <row r="16" ht="22" customHeight="1">
       <c r="B16" s="4" t="inlineStr">
         <is>
           <t>WriteWise</t>
@@ -1919,7 +1921,7 @@
         <v>46280</v>
       </c>
     </row>
-    <row r="17" ht="54" customHeight="1">
+    <row r="17" ht="22" customHeight="1">
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>ChronoBase</t>
@@ -2007,7 +2009,7 @@
         <v>46178</v>
       </c>
     </row>
-    <row r="18" ht="38" customHeight="1">
+    <row r="18" ht="22" customHeight="1">
       <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Kanbanly</t>
@@ -2091,7 +2093,7 @@
         <v>46264</v>
       </c>
     </row>
-    <row r="19" ht="38" customHeight="1">
+    <row r="19" ht="22" customHeight="1">
       <c r="B19" s="3" t="inlineStr">
         <is>
           <t>SummarEase</t>
@@ -2179,7 +2181,7 @@
         <v>46274</v>
       </c>
     </row>
-    <row r="20" ht="70" customHeight="1">
+    <row r="20" ht="22" customHeight="1">
       <c r="B20" s="4" t="inlineStr">
         <is>
           <t>WorkWhale</t>
@@ -2267,7 +2269,7 @@
         <v>46285</v>
       </c>
     </row>
-    <row r="21" ht="38" customHeight="1">
+    <row r="21" ht="22" customHeight="1">
       <c r="B21" s="3" t="inlineStr">
         <is>
           <t>GoalGrid</t>
@@ -2355,7 +2357,7 @@
         <v>46222</v>
       </c>
     </row>
-    <row r="22" ht="54" customHeight="1">
+    <row r="22" ht="22" customHeight="1">
       <c r="B22" s="4" t="inlineStr">
         <is>
           <t>AutoMateHQ</t>
@@ -2439,7 +2441,7 @@
         <v>46261</v>
       </c>
     </row>
-    <row r="23" ht="38" customHeight="1">
+    <row r="23" ht="22" customHeight="1">
       <c r="B23" s="3" t="inlineStr">
         <is>
           <t>ClientDesk</t>
@@ -2523,7 +2525,7 @@
         <v>46290</v>
       </c>
     </row>
-    <row r="24" ht="38" customHeight="1">
+    <row r="24" ht="22" customHeight="1">
       <c r="B24" s="4" t="inlineStr">
         <is>
           <t>SprintBoard</t>
@@ -2608,7 +2610,7 @@
       </c>
     </row>
     <row r="25" ht="22" customHeight="1"/>
-    <row r="26" ht="86" customHeight="1">
+    <row r="26" ht="22" customHeight="1">
       <c r="B26" s="5" t="inlineStr">
         <is>
           <t>Concept Project — all companies, prices, and sources are fictional demo data. Confidence: High / Medium / Needs verification.</t>
@@ -2631,14 +2633,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R28"/>
+  <dimension ref="B2:R28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="27" customWidth="1" min="5" max="5"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
     <col width="28" customWidth="1" min="6" max="6"/>
     <col width="28" customWidth="1" min="7" max="7"/>
     <col width="28" customWidth="1" min="8" max="8"/>
@@ -2650,8 +2652,8 @@
     <col width="28" customWidth="1" min="14" max="14"/>
     <col width="28" customWidth="1" min="15" max="15"/>
     <col width="28" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="26" customWidth="1" min="18" max="18"/>
+    <col width="15" customWidth="1" min="17" max="17"/>
+    <col width="28" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -2750,7 +2752,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="86" customHeight="1">
+    <row r="5" ht="22" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
           <t>R01</t>
@@ -2837,7 +2839,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="86" customHeight="1">
+    <row r="6" ht="22" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
           <t>R02</t>
@@ -2920,7 +2922,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="70" customHeight="1">
+    <row r="7" ht="22" customHeight="1">
       <c r="B7" s="3" t="inlineStr">
         <is>
           <t>R03</t>
@@ -3007,7 +3009,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="54" customHeight="1">
+    <row r="8" ht="22" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
           <t>R04</t>
@@ -3094,7 +3096,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="54" customHeight="1">
+    <row r="9" ht="22" customHeight="1">
       <c r="B9" s="3" t="inlineStr">
         <is>
           <t>R05</t>
@@ -3173,7 +3175,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="54" customHeight="1">
+    <row r="10" ht="22" customHeight="1">
       <c r="B10" s="4" t="inlineStr">
         <is>
           <t>R06</t>
@@ -3260,7 +3262,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="38" customHeight="1">
+    <row r="11" ht="22" customHeight="1">
       <c r="B11" s="3" t="inlineStr">
         <is>
           <t>R07</t>
@@ -3343,7 +3345,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="38" customHeight="1">
+    <row r="12" ht="22" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
           <t>R08</t>
@@ -3430,7 +3432,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="38" customHeight="1">
+    <row r="13" ht="22" customHeight="1">
       <c r="B13" s="3" t="inlineStr">
         <is>
           <t>R09</t>
@@ -3513,7 +3515,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="38" customHeight="1">
+    <row r="14" ht="22" customHeight="1">
       <c r="B14" s="4" t="inlineStr">
         <is>
           <t>R10</t>
@@ -3596,7 +3598,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="38" customHeight="1">
+    <row r="15" ht="22" customHeight="1">
       <c r="B15" s="3" t="inlineStr">
         <is>
           <t>R11</t>
@@ -3683,7 +3685,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="38" customHeight="1">
+    <row r="16" ht="22" customHeight="1">
       <c r="B16" s="4" t="inlineStr">
         <is>
           <t>R12</t>
@@ -3766,7 +3768,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="38" customHeight="1">
+    <row r="17" ht="22" customHeight="1">
       <c r="B17" s="3" t="inlineStr">
         <is>
           <t>R13</t>
@@ -3853,7 +3855,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="38" customHeight="1">
+    <row r="18" ht="22" customHeight="1">
       <c r="B18" s="4" t="inlineStr">
         <is>
           <t>R14</t>
@@ -3936,7 +3938,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="38" customHeight="1">
+    <row r="19" ht="22" customHeight="1">
       <c r="B19" s="3" t="inlineStr">
         <is>
           <t>R15</t>
@@ -4019,7 +4021,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="54" customHeight="1">
+    <row r="20" ht="22" customHeight="1">
       <c r="B20" s="4" t="inlineStr">
         <is>
           <t>R16</t>
@@ -4106,7 +4108,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="38" customHeight="1">
+    <row r="21" ht="22" customHeight="1">
       <c r="B21" s="3" t="inlineStr">
         <is>
           <t>R17</t>
@@ -4193,7 +4195,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="54" customHeight="1">
+    <row r="22" ht="22" customHeight="1">
       <c r="B22" s="4" t="inlineStr">
         <is>
           <t>R18</t>
@@ -4276,7 +4278,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="38" customHeight="1">
+    <row r="23" ht="22" customHeight="1">
       <c r="B23" s="3" t="inlineStr">
         <is>
           <t>R19</t>
@@ -4359,7 +4361,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="38" customHeight="1">
+    <row r="24" ht="22" customHeight="1">
       <c r="B24" s="4" t="inlineStr">
         <is>
           <t>R20</t>
@@ -4442,7 +4444,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="70" customHeight="1">
+    <row r="25" ht="22" customHeight="1">
       <c r="B25" s="3" t="inlineStr">
         <is>
           <t>R21</t>
@@ -4517,7 +4519,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="38" customHeight="1">
+    <row r="26" ht="22" customHeight="1">
       <c r="B26" s="4" t="inlineStr">
         <is>
           <t>R22</t>
@@ -4585,7 +4587,7 @@
       </c>
     </row>
     <row r="27" ht="22" customHeight="1"/>
-    <row r="28" ht="118" customHeight="1">
+    <row r="28" ht="22" customHeight="1">
       <c r="B28" s="5" t="inlineStr">
         <is>
           <t>Records R21 and R22 duplicate R01 and R02 under variant names — merged during cleaning. Formatting inconsistencies are intentional (demonstration data).</t>
@@ -4608,16 +4610,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="B2:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
     <col width="48" customWidth="1" min="4" max="4"/>
     <col width="48" customWidth="1" min="5" max="5"/>
     <col width="48" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="15" customHeight="1"/>
@@ -4661,7 +4663,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="70" customHeight="1">
+    <row r="5" ht="22" customHeight="1">
       <c r="B5" s="13" t="n">
         <v>1</v>
       </c>
@@ -4693,7 +4695,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="54" customHeight="1">
+    <row r="6" ht="22" customHeight="1">
       <c r="B6" s="14" t="n">
         <v>2</v>
       </c>
@@ -4724,7 +4726,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="54" customHeight="1">
+    <row r="7" ht="22" customHeight="1">
       <c r="B7" s="13" t="n">
         <v>3</v>
       </c>
@@ -4755,7 +4757,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="38" customHeight="1">
+    <row r="8" ht="22" customHeight="1">
       <c r="B8" s="14" t="n">
         <v>4</v>
       </c>
@@ -4785,7 +4787,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="70" customHeight="1">
+    <row r="9" ht="22" customHeight="1">
       <c r="B9" s="13" t="n">
         <v>5</v>
       </c>
@@ -4816,7 +4818,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="54" customHeight="1">
+    <row r="10" ht="22" customHeight="1">
       <c r="B10" s="14" t="n">
         <v>6</v>
       </c>
@@ -4847,7 +4849,7 @@
       </c>
     </row>
     <row r="11" ht="22" customHeight="1"/>
-    <row r="12" ht="294" customHeight="1">
+    <row r="12" ht="22" customHeight="1">
       <c r="B12" s="5" t="inlineStr">
         <is>
           <t>Every transformation in this log is reproducible: raw record IDs reference the Raw Data sheet.</t>
@@ -4869,12 +4871,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D64"/>
+  <dimension ref="B2:D64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
@@ -5003,14 +5005,14 @@
       </c>
     </row>
     <row r="14" ht="22" customHeight="1"/>
-    <row r="15" ht="26" customHeight="1">
+    <row r="15" ht="22" customHeight="1">
       <c r="B15" s="15" t="inlineStr">
         <is>
           <t>Products by Category</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="28" customHeight="1">
+    <row r="16" ht="22" customHeight="1">
       <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Product category</t>
@@ -5132,14 +5134,14 @@
       </c>
     </row>
     <row r="25" ht="22" customHeight="1"/>
-    <row r="26" ht="26" customHeight="1">
+    <row r="26" ht="22" customHeight="1">
       <c r="B26" s="15" t="inlineStr">
         <is>
           <t>Starting Price Distribution</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="28" customHeight="1">
+    <row r="27" ht="22" customHeight="1">
       <c r="B27" s="2" t="inlineStr">
         <is>
           <t>Price band (USD/user/mo)</t>
@@ -5209,14 +5211,14 @@
       </c>
     </row>
     <row r="32" ht="22" customHeight="1"/>
-    <row r="33" ht="26" customHeight="1">
+    <row r="33" ht="22" customHeight="1">
       <c r="B33" s="15" t="inlineStr">
         <is>
           <t>Price Statistics</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="28" customHeight="1">
+    <row r="34" ht="22" customHeight="1">
       <c r="B34" s="2" t="inlineStr">
         <is>
           <t>Statistic</t>
@@ -5277,14 +5279,14 @@
       </c>
     </row>
     <row r="39" ht="22" customHeight="1"/>
-    <row r="40" ht="26" customHeight="1">
+    <row r="40" ht="22" customHeight="1">
       <c r="B40" s="15" t="inlineStr">
         <is>
           <t>Free Plan Availability</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="28" customHeight="1">
+    <row r="41" ht="22" customHeight="1">
       <c r="B41" s="2" t="inlineStr">
         <is>
           <t>Availability</t>
@@ -5341,14 +5343,14 @@
       </c>
     </row>
     <row r="45" ht="22" customHeight="1"/>
-    <row r="46" ht="26" customHeight="1">
+    <row r="46" ht="22" customHeight="1">
       <c r="B46" s="15" t="inlineStr">
         <is>
           <t>AI Feature Adoption</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="28" customHeight="1">
+    <row r="47" ht="22" customHeight="1">
       <c r="B47" s="2" t="inlineStr">
         <is>
           <t>AI features</t>
@@ -5392,14 +5394,14 @@
       </c>
     </row>
     <row r="50" ht="22" customHeight="1"/>
-    <row r="51" ht="26" customHeight="1">
+    <row r="51" ht="22" customHeight="1">
       <c r="B51" s="15" t="inlineStr">
         <is>
           <t>Target Customer Distribution</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="28" customHeight="1">
+    <row r="52" ht="22" customHeight="1">
       <c r="B52" s="2" t="inlineStr">
         <is>
           <t>Target customer</t>
@@ -5469,14 +5471,14 @@
       </c>
     </row>
     <row r="57" ht="22" customHeight="1"/>
-    <row r="58" ht="26" customHeight="1">
+    <row r="58" ht="22" customHeight="1">
       <c r="B58" s="15" t="inlineStr">
         <is>
           <t>Data Confidence</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="28" customHeight="1">
+    <row r="59" ht="22" customHeight="1">
       <c r="B59" s="2" t="inlineStr">
         <is>
           <t>Confidence level</t>
@@ -5533,7 +5535,7 @@
       </c>
     </row>
     <row r="63" ht="22" customHeight="1"/>
-    <row r="64" ht="54" customHeight="1">
+    <row r="64" ht="22" customHeight="1">
       <c r="B64" s="5" t="inlineStr">
         <is>
           <t>All figures derived from the Clean Data sheet. Concept Project — fictional demo data.</t>
@@ -5563,12 +5565,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="B2:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="43" customWidth="1" min="3" max="3"/>
+    <col width="47" customWidth="1" min="3" max="3"/>
     <col width="52" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
@@ -5604,7 +5606,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="38" customHeight="1">
+    <row r="5" ht="22" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Source recorded</t>
@@ -5626,7 +5628,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="54" customHeight="1">
+    <row r="6" ht="22" customHeight="1">
       <c r="B6" s="4" t="inlineStr">
         <is>
           <t>Duplicate checked</t>
@@ -5648,7 +5650,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="54" customHeight="1">
+    <row r="7" ht="22" customHeight="1">
       <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Pricing normalized</t>
@@ -5670,7 +5672,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="38" customHeight="1">
+    <row r="8" ht="22" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
           <t>Missing values flagged</t>
@@ -5692,7 +5694,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="54" customHeight="1">
+    <row r="9" ht="22" customHeight="1">
       <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Unclear claims marked for verification</t>
@@ -5714,7 +5716,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="38" customHeight="1">
+    <row r="10" ht="22" customHeight="1">
       <c r="B10" s="4" t="inlineStr">
         <is>
           <t>No unsupported assumptions</t>
@@ -5736,7 +5738,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="38" customHeight="1">
+    <row r="11" ht="22" customHeight="1">
       <c r="B11" s="3" t="inlineStr">
         <is>
           <t>Dates standardized</t>
@@ -5758,7 +5760,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="38" customHeight="1">
+    <row r="12" ht="22" customHeight="1">
       <c r="B12" s="4" t="inlineStr">
         <is>
           <t>Final manual review completed</t>
@@ -5781,7 +5783,7 @@
       </c>
     </row>
     <row r="13" ht="22" customHeight="1"/>
-    <row r="14" ht="38" customHeight="1">
+    <row r="14" ht="22" customHeight="1">
       <c r="B14" s="5" t="inlineStr">
         <is>
           <t>Quality process mirrors what would be used on a live client engagement.</t>

</xml_diff>